<commit_message>
Added support for time-series in the summary string in the environment panel Updated the path to the R distribution for the test framework Added a test TestTimeSeriesSummary to the SummaryTests Updated the RScript.Evaluate function to accept EvalOptions instead of a T/F SuppressOutput parameter. EvalOptions can be one of (case insensitive) 'SuppressOutput', 'DataFrame' (or 'df' shorthand), 'List' ('ls' shorthand) or 'NamedVector' ('nv' shorthand). Updated the RScript.Function to allow the return value to be optional. Added support for EvalOptions as above. Updated the vector output to include the 'names' in the first column if they are present; i.e. this is a 'named' vector. Updated the version number: 2.0.0.0 and the AssemblyCopyright to 2026 Added the facility to pass in a single parameter (rather than a parameter block of key = value). This makes it easier somewhat easier to write scripts:  =RScript.Evaluate("adf.test("&C4&")") vs =RScript.Function(,"adf.test","model")
</commit_message>
<xml_diff>
--- a/ExcelRAddIn/Tests/AddIn Test.xlsx
+++ b/ExcelRAddIn/Tests/AddIn Test.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Development\Projects\C#\Office\Office365 AddIns\ExcelRAddIn\Tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C9F1BB9-9693-44C7-9B0B-4C5B85D50B20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDC442AF-79BB-4C42-A85C-B1D69E31434E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{0F2AA292-504D-47F7-886F-362165F7C2B7}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{0F2AA292-504D-47F7-886F-362165F7C2B7}"/>
   </bookViews>
   <sheets>
     <sheet name="Linear Model" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
   <si>
     <t>fm</t>
   </si>
@@ -198,6 +198,12 @@
   </si>
   <si>
     <t>=RScript.Evaluate(B90)</t>
+  </si>
+  <si>
+    <t>summary(fm$residuals)</t>
+  </si>
+  <si>
+    <t>summary(fm)$coefficients</t>
   </si>
 </sst>
 </file>
@@ -814,7 +820,7 @@
         <v>1</v>
       </c>
       <c r="D3" s="6" t="str" cm="1">
-        <f t="array" ref="D3">_xll.RScript.Evaluate(B3, "true")</f>
+        <f t="array" ref="D3">_xll.RScript.Evaluate(B3, TRUE)</f>
         <v>OK</v>
       </c>
     </row>
@@ -864,10 +870,10 @@
       </c>
       <c r="E19" s="5" cm="1">
         <f t="array" ref="E19:F19">TRANSPOSE(_xll.RScript.Evaluate($B$19&amp;"$"&amp;D19))</f>
-        <v>7.8534553462568338E-2</v>
+        <v>8.3242921028025732E-2</v>
       </c>
       <c r="F19" s="5">
-        <v>9.6124662652678439E-2</v>
+        <v>-9.6405256536097425E-2</v>
       </c>
       <c r="G19" s="5"/>
       <c r="H19" s="5"/>
@@ -887,154 +893,154 @@
       </c>
       <c r="E20" s="5" cm="1">
         <f t="array" ref="E20:BB20">TRANSPOSE(_xll.RScript.Evaluate($B$19&amp;"$"&amp;D20))</f>
-        <v>0.14544475288926215</v>
+        <v>-0.22552153148627149</v>
       </c>
       <c r="F20" s="5">
-        <v>1.6982297065551539</v>
+        <v>1.2962435052866932</v>
       </c>
       <c r="G20" s="5">
-        <v>-0.32826482498224052</v>
+        <v>-0.70252823975309198</v>
       </c>
       <c r="H20" s="5">
-        <v>-2.1263388022976604</v>
+        <v>0.2271591889602437</v>
       </c>
       <c r="I20" s="5">
-        <v>-0.87651741598721566</v>
+        <v>3.6046560105801595E-2</v>
       </c>
       <c r="J20" s="5">
-        <v>0.26318630558144473</v>
+        <v>-0.41442956020325017</v>
       </c>
       <c r="K20" s="5">
-        <v>2.3182085031953807</v>
+        <v>-1.0657923631907413</v>
       </c>
       <c r="L20" s="5">
-        <v>0.88751133590512266</v>
+        <v>-0.44830921413214392</v>
       </c>
       <c r="M20" s="5">
-        <v>0.60408830355245069</v>
+        <v>-0.33672444710775457</v>
       </c>
       <c r="N20" s="5">
-        <v>-1.8503657907532607</v>
+        <v>-0.18045642509137724</v>
       </c>
       <c r="O20" s="5">
-        <v>-0.64774056473127894</v>
+        <v>0.35808251340620811</v>
       </c>
       <c r="P20" s="5">
-        <v>-0.32899910093210705</v>
+        <v>-2.4805536602539226E-2</v>
       </c>
       <c r="Q20" s="5">
-        <v>-7.2617769708340385E-2</v>
+        <v>0.91759605676943956</v>
       </c>
       <c r="R20">
-        <v>0.41557834837444713</v>
+        <v>1.0447527997306805</v>
       </c>
       <c r="S20">
-        <v>-0.69404440468102579</v>
+        <v>0.90328219866046544</v>
       </c>
       <c r="T20">
-        <v>0.87292246234179305</v>
+        <v>-1.0003298840221302</v>
       </c>
       <c r="U20">
-        <v>0.17606659375262068</v>
+        <v>-0.85496882294234045</v>
       </c>
       <c r="V20">
-        <v>0.14704321192089187</v>
+        <v>1.0838993404476023</v>
       </c>
       <c r="W20">
-        <v>-0.58658013906890016</v>
+        <v>-0.37039485846668313</v>
       </c>
       <c r="X20">
-        <v>-0.20332186483209674</v>
+        <v>1.6441216771114937</v>
       </c>
       <c r="Y20">
-        <v>-0.96859311945873572</v>
+        <v>0.96936248202816677</v>
       </c>
       <c r="Z20">
-        <v>0.46436704683775254</v>
+        <v>0.13073483019304741</v>
       </c>
       <c r="AA20">
-        <v>0.87644553418109372</v>
+        <v>-1.2945693122605377</v>
       </c>
       <c r="AB20">
-        <v>0.83831405512318524</v>
+        <v>0.30423320151994881</v>
       </c>
       <c r="AC20">
-        <v>-0.44561099332094889</v>
+        <v>0.3159317783707839</v>
       </c>
       <c r="AD20">
-        <v>-0.67254861386887654</v>
+        <v>-0.37845517924634153</v>
       </c>
       <c r="AE20">
-        <v>-0.22146361163709904</v>
+        <v>-0.33171287355208678</v>
       </c>
       <c r="AF20">
-        <v>0.85768863450376076</v>
+        <v>-1.7095233446968484E-3</v>
       </c>
       <c r="AG20">
-        <v>-0.48829184760834998</v>
+        <v>0.4063209044544448</v>
       </c>
       <c r="AH20">
-        <v>4.4391245049364758E-2</v>
+        <v>0.57771268753014371</v>
       </c>
       <c r="AI20">
-        <v>0.1971529390979154</v>
+        <v>-0.60172106293651229</v>
       </c>
       <c r="AJ20">
-        <v>0.6067457769548793</v>
+        <v>0.50724591949851416</v>
       </c>
       <c r="AK20">
-        <v>-2.0336075302121368</v>
+        <v>1.2787823180033371</v>
       </c>
       <c r="AL20">
-        <v>0.12931593861011187</v>
+        <v>-0.2527007172993363</v>
       </c>
       <c r="AM20">
-        <v>-0.43457594147347955</v>
+        <v>-0.61370926380585566</v>
       </c>
       <c r="AN20">
-        <v>-0.9053138934939321</v>
+        <v>-0.61370949899814475</v>
       </c>
       <c r="AO20">
-        <v>-0.38687570965990892</v>
+        <v>-1.0131896111242278</v>
       </c>
       <c r="AP20">
-        <v>-1.4643899612306777</v>
+        <v>0.66203049831477001</v>
       </c>
       <c r="AQ20">
-        <v>0.42431191702343007</v>
+        <v>-1.5610740329308124</v>
       </c>
       <c r="AR20">
-        <v>-0.46362526515927061</v>
+        <v>-1.3236520540464263</v>
       </c>
       <c r="AS20">
-        <v>0.11025073607485925</v>
+        <v>-0.22164474475888163</v>
       </c>
       <c r="AT20">
-        <v>0.84893983710431065</v>
+        <v>0.72632694382389928</v>
       </c>
       <c r="AU20">
-        <v>-1.6706344201214827</v>
+        <v>-2.6404000861640959</v>
       </c>
       <c r="AV20">
-        <v>0.59090941579041489</v>
+        <v>0.39116241160745824</v>
       </c>
       <c r="AW20">
-        <v>1.0954397281243871</v>
+        <v>0.59967123959794133</v>
       </c>
       <c r="AX20">
-        <v>-0.49642401572781303</v>
+        <v>0.70162069464980725</v>
       </c>
       <c r="AY20">
-        <v>0.65426510278509531</v>
+        <v>1.1487103232086107</v>
       </c>
       <c r="AZ20">
-        <v>1.2512922596446669</v>
+        <v>0.54963781306587467</v>
       </c>
       <c r="BA20">
-        <v>2.2548640784614786</v>
+        <v>-1.7436700988940606E-2</v>
       </c>
       <c r="BB20">
-        <v>-0.40622816848843513</v>
+        <v>-0.29072234189015533</v>
       </c>
     </row>
     <row r="21" spans="2:55" x14ac:dyDescent="0.3">
@@ -1043,154 +1049,154 @@
       </c>
       <c r="E21" s="5" cm="1">
         <f t="array" ref="E21:BB21">TRANSPOSE(_xll.RScript.Evaluate($B$19&amp;"$"&amp;D21))</f>
-        <v>-0.6827468611324834</v>
+        <v>-0.54506832041362485</v>
       </c>
       <c r="F21" s="5">
-        <v>-0.71156110085390267</v>
+        <v>0.75700405433530571</v>
       </c>
       <c r="G21" s="5">
-        <v>-0.23486717465009313</v>
+        <v>-0.62028195228393501</v>
       </c>
       <c r="H21" s="5">
-        <v>-1.841353000609091</v>
+        <v>0.42000020623275147</v>
       </c>
       <c r="I21" s="5">
-        <v>-0.94806560779494964</v>
+        <v>0.16184923817874808</v>
       </c>
       <c r="J21" s="5">
-        <v>0.5056090314138314</v>
+        <v>-0.26875403625161359</v>
       </c>
       <c r="K21" s="5">
-        <v>2.1918852482433597</v>
+        <v>-1.1557700876163095</v>
       </c>
       <c r="L21" s="5">
-        <v>1.0088723016391516</v>
+        <v>-0.43765751657230628</v>
       </c>
       <c r="M21" s="5">
-        <v>0.62232895708882741</v>
+        <v>-9.8646481674696848E-2</v>
       </c>
       <c r="N21" s="5">
-        <v>-2.0501698015596634</v>
+        <v>0.18003721199625167</v>
       </c>
       <c r="O21" s="5">
-        <v>-0.3904448589628417</v>
+        <v>0.61921866680711257</v>
       </c>
       <c r="P21" s="5">
-        <v>-0.11671821732861376</v>
+        <v>0.10558747083760185</v>
       </c>
       <c r="Q21" s="5">
-        <v>-0.48539339439008333</v>
+        <v>0.82331492323910926</v>
       </c>
       <c r="R21">
-        <v>0.21956368107900276</v>
+        <v>0.87723946937583475</v>
       </c>
       <c r="S21">
-        <v>-0.69610552679029991</v>
+        <v>0.90472543513738568</v>
       </c>
       <c r="T21">
-        <v>0.65172711225956159</v>
+        <v>-0.9746273444249578</v>
       </c>
       <c r="U21">
-        <v>0.18462401469150699</v>
+        <v>-0.832361674545403</v>
       </c>
       <c r="V21">
-        <v>3.0468084295907166E-2</v>
+        <v>1.3970943199101735</v>
       </c>
       <c r="W21">
-        <v>-0.37218878164786429</v>
+        <v>-0.37688710240234702</v>
       </c>
       <c r="X21">
-        <v>-2.68290708017207E-2</v>
+        <v>1.5364524391461674</v>
       </c>
       <c r="Y21">
-        <v>-1.1053124237835832</v>
+        <v>0.9734613767565935</v>
       </c>
       <c r="Z21">
-        <v>4.1084916371791458E-2</v>
+        <v>-2.5134652315396411E-4</v>
       </c>
       <c r="AA21">
-        <v>0.69534383285897117</v>
+        <v>-1.5049487064877205</v>
       </c>
       <c r="AB21">
-        <v>0.53180775926345514</v>
+        <v>0.19529899075302376</v>
       </c>
       <c r="AC21">
-        <v>-0.52805137621320064</v>
+        <v>0.63631039447922988</v>
       </c>
       <c r="AD21">
-        <v>-0.61849582633564293</v>
+        <v>-0.48525733501397861</v>
       </c>
       <c r="AE21">
-        <v>-0.55883425812934873</v>
+        <v>-0.61393555620982843</v>
       </c>
       <c r="AF21">
-        <v>0.86607087348170375</v>
+        <v>-3.6941017736278427E-2</v>
       </c>
       <c r="AG21">
-        <v>-0.70265930618851868</v>
+        <v>0.56143640832985742</v>
       </c>
       <c r="AH21">
-        <v>-0.52334636838775495</v>
+        <v>0.42566744754594998</v>
       </c>
       <c r="AI21">
-        <v>0.41521611494262145</v>
+        <v>-0.51977906836144461</v>
       </c>
       <c r="AJ21">
-        <v>0.59036443317929133</v>
+        <v>0.76370751027897299</v>
       </c>
       <c r="AK21">
-        <v>-1.8965039322908157</v>
+        <v>1.6020939485939925</v>
       </c>
       <c r="AL21">
-        <v>4.9252187037200343E-2</v>
+        <v>-0.38863074795826119</v>
       </c>
       <c r="AM21">
-        <v>-0.61196996669774384</v>
+        <v>-0.62499124191055955</v>
       </c>
       <c r="AN21">
-        <v>-0.77034984013139596</v>
+        <v>-0.83085552778222282</v>
       </c>
       <c r="AO21">
-        <v>-0.4006044206932905</v>
+        <v>-0.93302108520339477</v>
       </c>
       <c r="AP21">
-        <v>-1.4816396827930642</v>
+        <v>0.8803533799795189</v>
       </c>
       <c r="AQ21">
-        <v>0.50335126447798739</v>
+        <v>-1.4180682163456459</v>
       </c>
       <c r="AR21">
-        <v>-0.26481003642400347</v>
+        <v>-1.1254341757370778</v>
       </c>
       <c r="AS21">
-        <v>0.59864364731009478</v>
+        <v>-0.3811788857845913</v>
       </c>
       <c r="AT21">
-        <v>0.78864857463271143</v>
+        <v>0.52271792052679078</v>
       </c>
       <c r="AU21">
-        <v>-1.5120302563481118</v>
+        <v>-2.4822513938178945</v>
       </c>
       <c r="AV21">
-        <v>0.6824941290487645</v>
+        <v>9.4128001547871237E-2</v>
       </c>
       <c r="AW21">
-        <v>1.3478801667830316</v>
+        <v>0.54073032831737111</v>
       </c>
       <c r="AX21">
-        <v>-0.6705697276385052</v>
+        <v>0.89473821660983122</v>
       </c>
       <c r="AY21">
-        <v>0.67639588334553569</v>
+        <v>1.1500416906597974</v>
       </c>
       <c r="AZ21">
-        <v>1.3135142737883081</v>
+        <v>0.68135861178892487</v>
       </c>
       <c r="BA21">
-        <v>2.7530611938643537</v>
+        <v>0.2435205212277074</v>
       </c>
       <c r="BB21">
-        <v>-1.1288802923744146</v>
+        <v>-0.51371264432622665</v>
       </c>
     </row>
     <row r="22" spans="2:55" x14ac:dyDescent="0.3">
@@ -1220,154 +1226,154 @@
       </c>
       <c r="E23" s="5" cm="1">
         <f t="array" ref="E23:BB23">TRANSPOSE(_xll.RScript.Evaluate($B$19&amp;"$"&amp;D23))</f>
-        <v>9.8595139996497966E-2</v>
+        <v>6.0070570598454082E-2</v>
       </c>
       <c r="F23" s="5">
-        <v>9.967615769743321E-2</v>
+        <v>1.1707043296273811E-2</v>
       </c>
       <c r="G23" s="5">
-        <v>4.9432457647497041E-2</v>
+        <v>0.10861539266185982</v>
       </c>
       <c r="H23" s="5">
-        <v>-3.2031342812206098E-2</v>
+        <v>0.17712385174462966</v>
       </c>
       <c r="I23" s="5">
-        <v>0.1195678761251423</v>
+        <v>0.13559661689179095</v>
       </c>
       <c r="J23" s="5">
-        <v>-1.3933407767941913E-2</v>
+        <v>0.14790695076718674</v>
       </c>
       <c r="K23" s="5">
-        <v>0.14285838121411709</v>
+        <v>1.9303662330258931E-3</v>
       </c>
       <c r="L23" s="5">
-        <v>3.7542380260337849E-2</v>
+        <v>6.4265765495433391E-2</v>
       </c>
       <c r="M23" s="5">
-        <v>8.1389416085553612E-2</v>
+        <v>0.20514610576701359</v>
       </c>
       <c r="N23" s="5">
-        <v>0.17410259746741352</v>
+        <v>0.28097710646251756</v>
       </c>
       <c r="O23" s="5">
-        <v>-2.0257439088112505E-2</v>
+        <v>0.21942961574734343</v>
       </c>
       <c r="P23" s="5">
-        <v>-1.1170148780997868E-3</v>
+        <v>0.13844011940034681</v>
       </c>
       <c r="Q23" s="5">
-        <v>0.26465870406111247</v>
+        <v>-7.3540208246469785E-4</v>
       </c>
       <c r="R23">
-        <v>0.17249135835129709</v>
+        <v>-4.6099453051389405E-2</v>
       </c>
       <c r="S23">
-        <v>9.0021786033620987E-2</v>
+        <v>5.8561538174329963E-2</v>
       </c>
       <c r="T23">
-        <v>0.18319825281976421</v>
+        <v>7.3589084949347683E-2</v>
       </c>
       <c r="U23">
-        <v>8.550675279214015E-2</v>
+        <v>7.1671629372906387E-2</v>
       </c>
       <c r="V23">
-        <v>0.13871345109289956</v>
+        <v>0.2516777161901429</v>
       </c>
       <c r="W23">
-        <v>-2.014394056981561E-3</v>
+        <v>5.3645865102798396E-2</v>
       </c>
       <c r="X23">
-        <v>1.4100177663179475E-2</v>
+        <v>-9.028730403910501E-3</v>
       </c>
       <c r="Y23">
-        <v>0.14727880954270156</v>
+        <v>6.0206598974104519E-2</v>
       </c>
       <c r="Z23">
-        <v>0.26912609875475391</v>
+        <v>-2.3472524852254747E-2</v>
       </c>
       <c r="AA23">
-        <v>0.16615032485986281</v>
+        <v>-7.2653050931316798E-2</v>
       </c>
       <c r="AB23">
-        <v>0.21947269784490431</v>
+        <v>-9.8123241391023241E-3</v>
       </c>
       <c r="AC23">
-        <v>0.12419926525226738</v>
+        <v>0.25612765587618824</v>
       </c>
       <c r="AD23">
-        <v>6.6161999790227743E-2</v>
+        <v>-8.4916119953984404E-3</v>
       </c>
       <c r="AE23">
-        <v>0.23259630326332281</v>
+        <v>-0.11715673564186468</v>
       </c>
       <c r="AF23">
-        <v>8.5581240636035338E-2</v>
+        <v>3.5843192521296613E-2</v>
       </c>
       <c r="AG23">
-        <v>0.18029501487448152</v>
+        <v>0.1537545935933875</v>
       </c>
       <c r="AH23">
-        <v>0.3305489610599503</v>
+        <v>-3.651766702839665E-2</v>
       </c>
       <c r="AI23">
-        <v>-3.575661187920548E-3</v>
+        <v>0.10842689690513646</v>
       </c>
       <c r="AJ23">
-        <v>9.6110783041547077E-2</v>
+        <v>0.21653393452833714</v>
       </c>
       <c r="AK23">
-        <v>3.084857044936351E-2</v>
+        <v>0.25794452638168974</v>
       </c>
       <c r="AL23">
-        <v>0.12318871518330804</v>
+        <v>-2.6535019929086134E-2</v>
       </c>
       <c r="AM23">
-        <v>0.16457381094881601</v>
+        <v>5.06788402913948E-2</v>
       </c>
       <c r="AN23">
-        <v>3.1758310586096794E-2</v>
+        <v>-7.6844676585571592E-2</v>
       </c>
       <c r="AO23">
-        <v>9.4982876420630913E-2</v>
+        <v>0.10732831286818245</v>
       </c>
       <c r="AP23">
-        <v>9.648001962662045E-2</v>
+        <v>0.192908720220484</v>
       </c>
       <c r="AQ23">
-        <v>5.553764688951851E-2</v>
+        <v>0.14625318717280922</v>
       </c>
       <c r="AR23">
-        <v>4.608618014529775E-3</v>
+        <v>0.18045457523381492</v>
       </c>
       <c r="AS23">
-        <v>-0.1185205962805387</v>
+        <v>-4.1156704272665656E-2</v>
       </c>
       <c r="AT23">
-        <v>0.11478139930632347</v>
+        <v>-6.8459110761989517E-2</v>
       </c>
       <c r="AU23">
-        <v>2.1706471661199211E-2</v>
+        <v>0.15563351737764775</v>
       </c>
       <c r="AV23">
-        <v>5.0203323397702615E-2</v>
+        <v>-0.12633193433766837</v>
       </c>
       <c r="AW23">
-        <v>-1.819296637301826E-2</v>
+        <v>2.1156275525307966E-2</v>
       </c>
       <c r="AX23">
-        <v>0.16319261933684026</v>
+        <v>0.17729513395766616</v>
       </c>
       <c r="AY23">
-        <v>7.9735323546909709E-2</v>
+        <v>5.8492240346253332E-2</v>
       </c>
       <c r="AZ23">
-        <v>6.2688422526765875E-2</v>
+        <v>0.13926262635829489</v>
       </c>
       <c r="BA23">
-        <v>-0.12268937042614247</v>
+        <v>0.21931877592941482</v>
       </c>
       <c r="BB23">
-        <v>0.39641903015436442</v>
+        <v>-8.0464941159371917E-2</v>
       </c>
     </row>
     <row r="24" spans="2:55" x14ac:dyDescent="0.3">
@@ -1670,154 +1676,154 @@
         <v>y</v>
       </c>
       <c r="F31" s="5">
-        <v>0.24403989288576011</v>
+        <v>-0.16545096088781741</v>
       </c>
       <c r="G31" s="5">
-        <v>1.7979058642525871</v>
+        <v>1.307950548582967</v>
       </c>
       <c r="H31" s="5">
-        <v>-0.27883236733474348</v>
+        <v>-0.59391284709123215</v>
       </c>
       <c r="I31" s="5">
-        <v>-2.1583701451098665</v>
+        <v>0.40428304070487336</v>
       </c>
       <c r="J31" s="5">
-        <v>-0.75694953986207336</v>
+        <v>0.17164317699759254</v>
       </c>
       <c r="K31" s="5">
-        <v>0.24925289781350282</v>
+        <v>-0.26652260943606343</v>
       </c>
       <c r="L31" s="5">
-        <v>2.4610668844094978</v>
+        <v>-1.0638619969577154</v>
       </c>
       <c r="M31" s="5">
-        <v>0.9250537161654605</v>
+        <v>-0.38404344863671053</v>
       </c>
       <c r="N31" s="5">
-        <v>0.6854777196380043</v>
+        <v>-0.13157834134074098</v>
       </c>
       <c r="O31" s="5">
-        <v>-1.6762631932858472</v>
+        <v>0.1005206813711403</v>
       </c>
       <c r="P31" s="5">
-        <v>-0.66799800381939145</v>
+        <v>0.57751212915355155</v>
       </c>
       <c r="Q31" s="5">
-        <v>-0.33011611581020683</v>
+        <v>0.1136345827978076</v>
       </c>
       <c r="R31">
-        <v>0.19204093435277206</v>
+        <v>0.91686065468697486</v>
       </c>
       <c r="S31">
-        <v>0.58806970672574421</v>
+        <v>0.99865334667929107</v>
       </c>
       <c r="T31">
-        <v>-0.60402261864740481</v>
+        <v>0.9618437368347954</v>
       </c>
       <c r="U31">
-        <v>1.0561207151615573</v>
+        <v>-0.92674079907278251</v>
       </c>
       <c r="V31">
-        <v>0.26157334654476083</v>
+        <v>-0.78329719356943406</v>
       </c>
       <c r="W31">
-        <v>0.28575666301379143</v>
+        <v>1.3355770566377452</v>
       </c>
       <c r="X31">
-        <v>-0.58859453312588172</v>
+        <v>-0.31674899336388473</v>
       </c>
       <c r="Y31">
-        <v>-0.18922168716891727</v>
+        <v>1.6350929467075832</v>
       </c>
       <c r="Z31">
-        <v>-0.82131430991603416</v>
+        <v>1.0295690810022713</v>
       </c>
       <c r="AA31">
-        <v>0.73349314559250645</v>
+        <v>0.10726230534079266</v>
       </c>
       <c r="AB31">
-        <v>1.0425958590409565</v>
+        <v>-1.3672223631918545</v>
       </c>
       <c r="AC31">
-        <v>1.0577867529680895</v>
+        <v>0.29442087738084649</v>
       </c>
       <c r="AD31">
-        <v>-0.32141172806868151</v>
+        <v>0.57205943424697214</v>
       </c>
       <c r="AE31">
-        <v>-0.6063866140786488</v>
+        <v>-0.38694679124173997</v>
       </c>
       <c r="AF31">
-        <v>1.1132691626223755E-2</v>
+        <v>-0.44886960919395147</v>
       </c>
       <c r="AG31">
-        <v>0.9432698751397961</v>
+        <v>3.4133669176599768E-2</v>
       </c>
       <c r="AH31">
-        <v>-0.30799683273386846</v>
+        <v>0.5600754980478323</v>
       </c>
       <c r="AI31">
-        <v>0.37494020610931506</v>
+        <v>0.54119502050174706</v>
       </c>
       <c r="AJ31">
-        <v>0.19357727790999485</v>
+        <v>-0.49329416603137582</v>
       </c>
       <c r="AK31">
-        <v>0.70285655999642638</v>
+        <v>0.7237798540268513</v>
       </c>
       <c r="AL31">
-        <v>-2.0027589597627733</v>
+        <v>1.5367268443850268</v>
       </c>
       <c r="AM31">
-        <v>0.25250465379341991</v>
+        <v>-0.27923573722842243</v>
       </c>
       <c r="AN31">
-        <v>-0.27000213052466354</v>
+        <v>-0.56303042351446086</v>
       </c>
       <c r="AO31">
-        <v>-0.8735555829078353</v>
+        <v>-0.69055417558371635</v>
       </c>
       <c r="AP31">
-        <v>-0.291892833239278</v>
+        <v>-0.90586129825604533</v>
       </c>
       <c r="AQ31">
-        <v>-1.3679099416040572</v>
+        <v>0.85493921853525401</v>
       </c>
       <c r="AR31">
-        <v>0.47984956391294858</v>
+        <v>-1.4148208457580032</v>
       </c>
       <c r="AS31">
-        <v>-0.45901664714474083</v>
+        <v>-1.1431974788126114</v>
       </c>
       <c r="AT31">
-        <v>-8.2698602056794513E-3</v>
+        <v>-0.26280144903154729</v>
       </c>
       <c r="AU31">
-        <v>0.96372123641063412</v>
+        <v>0.65786783306190977</v>
       </c>
       <c r="AV31">
-        <v>-1.6489279484602835</v>
+        <v>-2.4847665687864482</v>
       </c>
       <c r="AW31">
-        <v>0.64111273918811751</v>
+        <v>0.26483047726978987</v>
       </c>
       <c r="AX31">
-        <v>1.0772467617513688</v>
+        <v>0.6208275151232493</v>
       </c>
       <c r="AY31">
-        <v>-0.33323139639097277</v>
+        <v>0.87891582860747341</v>
       </c>
       <c r="AZ31">
-        <v>0.73400042633200502</v>
+        <v>1.207202563554864</v>
       </c>
       <c r="BA31">
-        <v>1.3139806821714328</v>
+        <v>0.68890043942416956</v>
       </c>
       <c r="BB31">
-        <v>2.1321747080353362</v>
+        <v>0.20188207494047422</v>
       </c>
       <c r="BC31">
-        <v>-9.8091383340707106E-3</v>
+        <v>-0.37118728304952725</v>
       </c>
     </row>
     <row r="32" spans="2:55" x14ac:dyDescent="0.3">
@@ -1825,154 +1831,154 @@
         <v>x</v>
       </c>
       <c r="F32" s="5">
-        <v>0.20869344016752428</v>
+        <v>0.24036397248624272</v>
       </c>
       <c r="G32" s="5">
-        <v>0.21993943751203449</v>
+        <v>0.74203295859667606</v>
       </c>
       <c r="H32" s="5">
-        <v>-0.3027536847668747</v>
+        <v>-0.26318556213097977</v>
       </c>
       <c r="I32" s="5">
-        <v>-1.1502344270822147</v>
+        <v>-0.97381547531541124</v>
       </c>
       <c r="J32" s="5">
-        <v>0.42687611618297483</v>
+        <v>-0.54305851926406312</v>
       </c>
       <c r="K32" s="5">
-        <v>-0.96195875937291031</v>
+        <v>-0.67075211521218769</v>
       </c>
       <c r="L32" s="5">
-        <v>0.66917090761572429</v>
+        <v>0.84344524060836412</v>
       </c>
       <c r="M32" s="5">
-        <v>-0.42644803186821123</v>
+        <v>0.19684772609351106</v>
       </c>
       <c r="N32" s="5">
-        <v>2.9699585353038991E-2</v>
+        <v>-1.264486907862157</v>
       </c>
       <c r="O32" s="5">
-        <v>0.99420940856932749</v>
+        <v>-2.0510726545336602</v>
       </c>
       <c r="P32" s="5">
-        <v>-1.0277486528888009</v>
+        <v>-1.4126480195436717</v>
       </c>
       <c r="Q32" s="5">
-        <v>-0.82862780625268107</v>
+        <v>-0.57255382492191564</v>
       </c>
       <c r="R32">
-        <v>1.9362788431420086</v>
+        <v>0.87109693109987252</v>
       </c>
       <c r="S32">
-        <v>0.97744743436153636</v>
+        <v>1.3416527140403887</v>
       </c>
       <c r="T32">
-        <v>0.11950348905315647</v>
+        <v>0.25601698227372316</v>
       </c>
       <c r="U32">
-        <v>1.0888329432725401</v>
+        <v>0.10013806742024849</v>
       </c>
       <c r="V32">
-        <v>7.2532887369020985E-2</v>
+        <v>0.12002760088903172</v>
       </c>
       <c r="W32">
-        <v>0.62605054696287576</v>
+        <v>-1.747153643007521</v>
       </c>
       <c r="X32">
-        <v>-0.83796338313916929</v>
+        <v>0.30700666113725067</v>
       </c>
       <c r="Y32">
-        <v>-0.67032095636273525</v>
+        <v>0.95712261703682633</v>
       </c>
       <c r="Z32">
-        <v>0.71515731949585737</v>
+        <v>0.23895296669114344</v>
       </c>
       <c r="AA32">
-        <v>1.9827538535124822</v>
+        <v>1.1069463400091937</v>
       </c>
       <c r="AB32">
-        <v>0.91148066458107035</v>
+        <v>1.6170899550583084</v>
       </c>
       <c r="AC32">
-        <v>1.4662017061280042</v>
+        <v>0.96525073954120999</v>
       </c>
       <c r="AD32">
-        <v>0.47505718646521183</v>
+        <v>-1.7933123261118915</v>
       </c>
       <c r="AE32">
-        <v>-0.12871362385994017</v>
+        <v>0.95155115311659022</v>
       </c>
       <c r="AF32">
-        <v>1.6027286395523341</v>
+        <v>2.0787212634495087</v>
       </c>
       <c r="AG32">
-        <v>7.3307796136861503E-2</v>
+        <v>0.4916716184348417</v>
       </c>
       <c r="AH32">
-        <v>1.0586301018251492</v>
+        <v>-0.73140900298273448</v>
       </c>
       <c r="AI32">
-        <v>2.6217455608449884</v>
+        <v>1.24226201308411</v>
       </c>
       <c r="AJ32">
-        <v>-0.85420549091727582</v>
+        <v>-0.2612303185737706</v>
       </c>
       <c r="AK32">
-        <v>0.18284828361360123</v>
+        <v>-1.3826114704689632</v>
       </c>
       <c r="AL32">
-        <v>-0.49608478924400329</v>
+        <v>-1.8121585028742679</v>
       </c>
       <c r="AM32">
-        <v>0.46454427499096668</v>
+        <v>1.1387132289410722</v>
       </c>
       <c r="AN32">
-        <v>0.89507994214896014</v>
+        <v>0.33778324861816933</v>
       </c>
       <c r="AO32">
-        <v>-0.48662061936680379</v>
+        <v>1.6605691781303973</v>
       </c>
       <c r="AP32">
-        <v>0.17111449345205379</v>
+        <v>-0.24983483998238559</v>
       </c>
       <c r="AQ32">
-        <v>0.18668950994286992</v>
+        <v>-1.137549996056445</v>
       </c>
       <c r="AR32">
-        <v>-0.23924043984573629</v>
+        <v>-0.65359782659973875</v>
       </c>
       <c r="AS32">
-        <v>-0.76906314579381829</v>
+        <v>-1.0083646649432447</v>
       </c>
       <c r="AT32">
-        <v>-2.049995748282774</v>
+        <v>1.2903821821594539</v>
       </c>
       <c r="AU32">
-        <v>0.37708164422614165</v>
+        <v>1.5735867238028953</v>
       </c>
       <c r="AV32">
-        <v>-0.59119148232230845</v>
+        <v>-0.75089885085795516</v>
       </c>
       <c r="AW32">
-        <v>-0.29473424699791345</v>
+        <v>2.1738944835152436</v>
       </c>
       <c r="AX32">
-        <v>-1.0062716181911204</v>
+        <v>0.64401722202222933</v>
       </c>
       <c r="AY32">
-        <v>0.88071118834676099</v>
+        <v>-0.97559216487769063</v>
       </c>
       <c r="AZ32">
-        <v>1.2491800243608223E-2</v>
+        <v>0.25673580021546666</v>
       </c>
       <c r="BA32">
-        <v>-0.16484979503187619</v>
+        <v>-0.58108558955282097</v>
       </c>
       <c r="BB32">
-        <v>-2.0933641620754653</v>
+        <v>-1.4114982915940648</v>
       </c>
       <c r="BC32">
-        <v>3.3070022605997496</v>
+        <v>1.6981217422112238</v>
       </c>
     </row>
     <row r="34" spans="2:54" x14ac:dyDescent="0.3">
@@ -2006,154 +2012,154 @@
       </c>
       <c r="E36" cm="1">
         <f t="array" ref="E36:BB36">TRANSPOSE(_xll.RScript.Evaluate($B$34&amp;"$"&amp;D36))</f>
-        <v>0.14544475288926215</v>
+        <v>-0.22552153148627149</v>
       </c>
       <c r="F36">
-        <v>1.6982297065551539</v>
+        <v>1.2962435052866932</v>
       </c>
       <c r="G36">
-        <v>-0.32826482498224052</v>
+        <v>-0.70252823975309198</v>
       </c>
       <c r="H36">
-        <v>-2.1263388022976604</v>
+        <v>0.2271591889602437</v>
       </c>
       <c r="I36">
-        <v>-0.87651741598721566</v>
+        <v>3.6046560105801595E-2</v>
       </c>
       <c r="J36">
-        <v>0.26318630558144473</v>
+        <v>-0.41442956020325017</v>
       </c>
       <c r="K36">
-        <v>2.3182085031953807</v>
+        <v>-1.0657923631907413</v>
       </c>
       <c r="L36">
-        <v>0.88751133590512266</v>
+        <v>-0.44830921413214392</v>
       </c>
       <c r="M36">
-        <v>0.60408830355245069</v>
+        <v>-0.33672444710775457</v>
       </c>
       <c r="N36">
-        <v>-1.8503657907532607</v>
+        <v>-0.18045642509137724</v>
       </c>
       <c r="O36">
-        <v>-0.64774056473127894</v>
+        <v>0.35808251340620811</v>
       </c>
       <c r="P36">
-        <v>-0.32899910093210705</v>
+        <v>-2.4805536602539226E-2</v>
       </c>
       <c r="Q36">
-        <v>-7.2617769708340385E-2</v>
+        <v>0.91759605676943956</v>
       </c>
       <c r="R36">
-        <v>0.41557834837444713</v>
+        <v>1.0447527997306805</v>
       </c>
       <c r="S36">
-        <v>-0.69404440468102579</v>
+        <v>0.90328219866046544</v>
       </c>
       <c r="T36">
-        <v>0.87292246234179305</v>
+        <v>-1.0003298840221302</v>
       </c>
       <c r="U36">
-        <v>0.17606659375262068</v>
+        <v>-0.85496882294234045</v>
       </c>
       <c r="V36">
-        <v>0.14704321192089187</v>
+        <v>1.0838993404476023</v>
       </c>
       <c r="W36">
-        <v>-0.58658013906890016</v>
+        <v>-0.37039485846668313</v>
       </c>
       <c r="X36">
-        <v>-0.20332186483209674</v>
+        <v>1.6441216771114937</v>
       </c>
       <c r="Y36">
-        <v>-0.96859311945873572</v>
+        <v>0.96936248202816677</v>
       </c>
       <c r="Z36">
-        <v>0.46436704683775254</v>
+        <v>0.13073483019304741</v>
       </c>
       <c r="AA36">
-        <v>0.87644553418109372</v>
+        <v>-1.2945693122605377</v>
       </c>
       <c r="AB36">
-        <v>0.83831405512318524</v>
+        <v>0.30423320151994881</v>
       </c>
       <c r="AC36">
-        <v>-0.44561099332094889</v>
+        <v>0.3159317783707839</v>
       </c>
       <c r="AD36">
-        <v>-0.67254861386887654</v>
+        <v>-0.37845517924634153</v>
       </c>
       <c r="AE36">
-        <v>-0.22146361163709904</v>
+        <v>-0.33171287355208678</v>
       </c>
       <c r="AF36">
-        <v>0.85768863450376076</v>
+        <v>-1.7095233446968484E-3</v>
       </c>
       <c r="AG36">
-        <v>-0.48829184760834998</v>
+        <v>0.4063209044544448</v>
       </c>
       <c r="AH36">
-        <v>4.4391245049364758E-2</v>
+        <v>0.57771268753014371</v>
       </c>
       <c r="AI36">
-        <v>0.1971529390979154</v>
+        <v>-0.60172106293651229</v>
       </c>
       <c r="AJ36">
-        <v>0.6067457769548793</v>
+        <v>0.50724591949851416</v>
       </c>
       <c r="AK36">
-        <v>-2.0336075302121368</v>
+        <v>1.2787823180033371</v>
       </c>
       <c r="AL36">
-        <v>0.12931593861011187</v>
+        <v>-0.2527007172993363</v>
       </c>
       <c r="AM36">
-        <v>-0.43457594147347955</v>
+        <v>-0.61370926380585566</v>
       </c>
       <c r="AN36">
-        <v>-0.9053138934939321</v>
+        <v>-0.61370949899814475</v>
       </c>
       <c r="AO36">
-        <v>-0.38687570965990892</v>
+        <v>-1.0131896111242278</v>
       </c>
       <c r="AP36">
-        <v>-1.4643899612306777</v>
+        <v>0.66203049831477001</v>
       </c>
       <c r="AQ36">
-        <v>0.42431191702343007</v>
+        <v>-1.5610740329308124</v>
       </c>
       <c r="AR36">
-        <v>-0.46362526515927061</v>
+        <v>-1.3236520540464263</v>
       </c>
       <c r="AS36">
-        <v>0.11025073607485925</v>
+        <v>-0.22164474475888163</v>
       </c>
       <c r="AT36">
-        <v>0.84893983710431065</v>
+        <v>0.72632694382389928</v>
       </c>
       <c r="AU36">
-        <v>-1.6706344201214827</v>
+        <v>-2.6404000861640959</v>
       </c>
       <c r="AV36">
-        <v>0.59090941579041489</v>
+        <v>0.39116241160745824</v>
       </c>
       <c r="AW36">
-        <v>1.0954397281243871</v>
+        <v>0.59967123959794133</v>
       </c>
       <c r="AX36">
-        <v>-0.49642401572781303</v>
+        <v>0.70162069464980725</v>
       </c>
       <c r="AY36">
-        <v>0.65426510278509531</v>
+        <v>1.1487103232086107</v>
       </c>
       <c r="AZ36">
-        <v>1.2512922596446669</v>
+        <v>0.54963781306587467</v>
       </c>
       <c r="BA36">
-        <v>2.2548640784614786</v>
+        <v>-1.7436700988940606E-2</v>
       </c>
       <c r="BB36">
-        <v>-0.40622816848843513</v>
+        <v>-0.29072234189015533</v>
       </c>
     </row>
     <row r="37" spans="2:54" x14ac:dyDescent="0.3">
@@ -2184,7 +2190,7 @@
       </c>
       <c r="E39" cm="1">
         <f t="array" ref="E39">TRANSPOSE(_xll.RScript.Evaluate($B$34&amp;"$"&amp;D39))</f>
-        <v>0.97713512136322711</v>
+        <v>0.85537162902593444</v>
       </c>
       <c r="I39" s="1"/>
       <c r="R39" s="4"/>
@@ -2211,7 +2217,7 @@
       </c>
       <c r="E41" cm="1">
         <f t="array" ref="E41">TRANSPOSE(_xll.RScript.Evaluate($B$34&amp;"$"&amp;D41))</f>
-        <v>1.0927032743304671E-2</v>
+        <v>1.6055218390311911E-2</v>
       </c>
     </row>
     <row r="42" spans="2:54" x14ac:dyDescent="0.3">
@@ -2220,7 +2226,7 @@
       </c>
       <c r="E42" cm="1">
         <f t="array" ref="E42">TRANSPOSE(_xll.RScript.Evaluate($B$34&amp;"$"&amp;D42))</f>
-        <v>-9.6786540745430472E-3</v>
+        <v>-4.4436312265565547E-3</v>
       </c>
     </row>
     <row r="43" spans="2:54" x14ac:dyDescent="0.3">
@@ -2229,7 +2235,7 @@
       </c>
       <c r="E43" cm="1">
         <f t="array" ref="E43:G43">TRANSPOSE(_xll.RScript.Evaluate($B$34&amp;"$"&amp;D43))</f>
-        <v>0.53029209071740879</v>
+        <v>0.78322533656230497</v>
       </c>
       <c r="F43">
         <v>1</v>
@@ -2244,21 +2250,24 @@
       </c>
       <c r="E44" cm="1">
         <f t="array" ref="E44:F45">TRANSPOSE(_xll.RScript.Evaluate($B$34&amp;"$"&amp;D44))</f>
-        <v>2.0641366211616771E-2</v>
+        <v>2.0066186648894452E-2</v>
       </c>
       <c r="F44">
-        <v>-3.4211779848343422E-3</v>
+        <v>-1.0360666766140157E-3</v>
       </c>
     </row>
     <row r="45" spans="2:54" x14ac:dyDescent="0.3">
       <c r="E45">
-        <v>-3.4211779848343422E-3</v>
+        <v>-1.0360666766140157E-3</v>
       </c>
       <c r="F45">
-        <v>1.824926008248905E-2</v>
+        <v>1.6218288375678378E-2</v>
       </c>
     </row>
     <row r="47" spans="2:54" x14ac:dyDescent="0.3">
+      <c r="B47" t="s">
+        <v>46</v>
+      </c>
       <c r="D47" t="str" cm="1">
         <f t="array" ref="D47:F53">_xll.RScript.Evaluate(B35)</f>
         <v>Index</v>
@@ -2269,6 +2278,11 @@
       <c r="F47" t="str">
         <v>Freq</v>
       </c>
+      <c r="H47" t="str" cm="1">
+        <f t="array" ref="H47">_xll.RScript.Evaluate(B47,"DataFrame")</f>
+        <v xml:space="preserve">Exception: Error in dimnames(x) &lt;- dnx : 'dimnames' applied to non-array
+</v>
+      </c>
     </row>
     <row r="48" spans="2:54" x14ac:dyDescent="0.3">
       <c r="D48" t="str">
@@ -2278,10 +2292,10 @@
         <v>Min.</v>
       </c>
       <c r="F48">
-        <v>-2.1263388022976604</v>
-      </c>
-    </row>
-    <row r="49" spans="2:10" x14ac:dyDescent="0.3">
+        <v>-2.6404000861640959</v>
+      </c>
+    </row>
+    <row r="49" spans="2:15" x14ac:dyDescent="0.3">
       <c r="D49" t="str">
         <v>2</v>
       </c>
@@ -2289,10 +2303,10 @@
         <v>1st Qu.</v>
       </c>
       <c r="F49">
-        <v>-0.49439097369794727</v>
-      </c>
-    </row>
-    <row r="50" spans="2:10" x14ac:dyDescent="0.3">
+        <v>-0.43983930064992049</v>
+      </c>
+    </row>
+    <row r="50" spans="2:15" x14ac:dyDescent="0.3">
       <c r="D50" t="str">
         <v>3</v>
       </c>
@@ -2300,10 +2314,10 @@
         <v>Median</v>
       </c>
       <c r="F50">
-        <v>7.7320990562112002E-2</v>
-      </c>
-    </row>
-    <row r="51" spans="2:10" x14ac:dyDescent="0.3">
+        <v>-9.5731121668187272E-3</v>
+      </c>
+    </row>
+    <row r="51" spans="2:15" x14ac:dyDescent="0.3">
       <c r="D51" t="str">
         <v>4</v>
       </c>
@@ -2311,10 +2325,10 @@
         <v>Mean</v>
       </c>
       <c r="F51">
-        <v>2.1103995287430344E-17</v>
-      </c>
-    </row>
-    <row r="52" spans="2:10" x14ac:dyDescent="0.3">
+        <v>1.2543134933484801E-17</v>
+      </c>
+    </row>
+    <row r="52" spans="2:15" x14ac:dyDescent="0.3">
       <c r="D52" t="str">
         <v>5</v>
       </c>
@@ -2322,10 +2336,10 @@
         <v>3rd Qu.</v>
       </c>
       <c r="F52">
-        <v>0.60608140860427218</v>
-      </c>
-    </row>
-    <row r="53" spans="2:10" x14ac:dyDescent="0.3">
+        <v>0.59418160158099198</v>
+      </c>
+    </row>
+    <row r="53" spans="2:15" x14ac:dyDescent="0.3">
       <c r="D53" t="str">
         <v>6</v>
       </c>
@@ -2333,10 +2347,10 @@
         <v>Max.</v>
       </c>
       <c r="F53">
-        <v>2.3182085031953807</v>
-      </c>
-    </row>
-    <row r="55" spans="2:10" x14ac:dyDescent="0.3">
+        <v>1.6441216771114937</v>
+      </c>
+    </row>
+    <row r="55" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B55" s="5" t="str">
         <f>"coef = round(as.data.frame("&amp;B34&amp;"$"&amp;D37&amp;"), 4)"</f>
         <v>coef = round(as.data.frame(summary(fm)$coefficients), 4)</v>
@@ -2361,42 +2375,91 @@
       <c r="I55" s="1" t="str">
         <v>Pr(&gt;|t|)</v>
       </c>
-    </row>
-    <row r="56" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="K55" t="str" cm="1">
+        <f t="array" ref="K55:O57">_xll.RScript.Evaluate(B56, "DataFrame")</f>
+        <v>Index</v>
+      </c>
+      <c r="L55" t="str">
+        <v>Estimate</v>
+      </c>
+      <c r="M55" t="str">
+        <v>Std. Error</v>
+      </c>
+      <c r="N55" t="str">
+        <v>t value</v>
+      </c>
+      <c r="O55" t="str">
+        <v>Pr(&gt;|t|)</v>
+      </c>
+    </row>
+    <row r="56" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="B56" t="s">
+        <v>47</v>
+      </c>
       <c r="E56" s="1" t="str">
         <v>(Intercept)</v>
       </c>
       <c r="F56">
-        <v>7.85E-2</v>
+        <v>8.3199999999999996E-2</v>
       </c>
       <c r="G56">
-        <v>0.1404</v>
+        <v>0.1212</v>
       </c>
       <c r="H56">
-        <v>0.55940000000000001</v>
+        <v>0.68700000000000006</v>
       </c>
       <c r="I56">
-        <v>0.57850000000000001</v>
-      </c>
-    </row>
-    <row r="57" spans="2:10" x14ac:dyDescent="0.3">
+        <v>0.49540000000000001</v>
+      </c>
+      <c r="K56" t="str">
+        <v>(Intercept)</v>
+      </c>
+      <c r="L56">
+        <v>8.3242921028025732E-2</v>
+      </c>
+      <c r="M56">
+        <v>0.12116781189599471</v>
+      </c>
+      <c r="N56">
+        <v>0.68700523452117723</v>
+      </c>
+      <c r="O56">
+        <v>0.49538539249663127</v>
+      </c>
+    </row>
+    <row r="57" spans="2:15" x14ac:dyDescent="0.3">
       <c r="E57" s="1" t="str">
         <v>x</v>
       </c>
       <c r="F57">
-        <v>9.6100000000000005E-2</v>
+        <v>-9.64E-2</v>
       </c>
       <c r="G57">
-        <v>0.13200000000000001</v>
+        <v>0.1089</v>
       </c>
       <c r="H57">
-        <v>0.72819999999999996</v>
+        <v>-0.88500000000000001</v>
       </c>
       <c r="I57">
-        <v>0.47</v>
-      </c>
-    </row>
-    <row r="59" spans="2:10" x14ac:dyDescent="0.3">
+        <v>0.38059999999999999</v>
+      </c>
+      <c r="K57" t="str">
+        <v>x</v>
+      </c>
+      <c r="L57">
+        <v>-9.6405256536097425E-2</v>
+      </c>
+      <c r="M57">
+        <v>0.10893246985625667</v>
+      </c>
+      <c r="N57">
+        <v>-0.88500019014817444</v>
+      </c>
+      <c r="O57">
+        <v>0.3805684851417751</v>
+      </c>
+    </row>
+    <row r="59" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B59" t="s">
         <v>5</v>
       </c>
@@ -2420,7 +2483,7 @@
         <v>Pr(&gt;F)</v>
       </c>
     </row>
-    <row r="60" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="60" spans="2:15" x14ac:dyDescent="0.3">
       <c r="E60" s="1" t="str">
         <v>x</v>
       </c>
@@ -2440,7 +2503,7 @@
         <v>0.54749204609353308</v>
       </c>
     </row>
-    <row r="61" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="61" spans="2:15" x14ac:dyDescent="0.3">
       <c r="E61" s="1" t="str">
         <v>Residuals</v>
       </c>
@@ -2460,7 +2523,7 @@
         <v/>
       </c>
     </row>
-    <row r="63" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="63" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B63" t="s">
         <v>2</v>
       </c>
@@ -2593,22 +2656,22 @@
     </row>
     <row r="6" spans="2:9" x14ac:dyDescent="0.2">
       <c r="D6" s="10">
-        <v>-2.1263388022976604</v>
+        <v>-2.6404000861640959</v>
       </c>
       <c r="E6" s="10">
-        <v>-0.49439097369794727</v>
+        <v>-0.43983930064992049</v>
       </c>
       <c r="F6" s="10">
-        <v>7.7320990562112002E-2</v>
+        <v>-9.5731121668187272E-3</v>
       </c>
       <c r="G6" s="9">
-        <v>2.1103995287430344E-17</v>
+        <v>1.2543134933484801E-17</v>
       </c>
       <c r="H6" s="10">
-        <v>0.60608140860427218</v>
+        <v>0.59418160158099198</v>
       </c>
       <c r="I6" s="10">
-        <v>2.3182085031953807</v>
+        <v>1.6441216771114937</v>
       </c>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.2">
@@ -2639,16 +2702,16 @@
         <v>(Intercept)</v>
       </c>
       <c r="E9" s="8">
-        <v>7.85E-2</v>
+        <v>8.3199999999999996E-2</v>
       </c>
       <c r="F9" s="8">
-        <v>0.1404</v>
+        <v>0.1212</v>
       </c>
       <c r="G9" s="8">
-        <v>0.55940000000000001</v>
+        <v>0.68700000000000006</v>
       </c>
       <c r="H9" s="8">
-        <v>0.57850000000000001</v>
+        <v>0.49540000000000001</v>
       </c>
       <c r="I9" s="8"/>
     </row>
@@ -2657,23 +2720,23 @@
         <v>x</v>
       </c>
       <c r="E10" s="8">
-        <v>9.6100000000000005E-2</v>
+        <v>-9.64E-2</v>
       </c>
       <c r="F10" s="10">
-        <v>0.13200000000000001</v>
+        <v>0.1089</v>
       </c>
       <c r="G10" s="8">
-        <v>0.72819999999999996</v>
+        <v>-0.88500000000000001</v>
       </c>
       <c r="H10" s="10">
-        <v>0.47</v>
+        <v>0.38059999999999999</v>
       </c>
       <c r="I10" s="8"/>
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B12" s="8" t="str">
         <f>"Residual standard error: "&amp;ROUND('Linear Model'!E39, 3)&amp;" on "&amp;'Linear Model'!E26&amp;" degrees of freedom"</f>
-        <v>Residual standard error: 0.977 on 48 degrees of freedom</v>
+        <v>Residual standard error: 0.855 on 48 degrees of freedom</v>
       </c>
       <c r="C12" s="8"/>
       <c r="D12" s="8"/>
@@ -2686,11 +2749,11 @@
     <row r="13" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B13" s="8" t="str">
         <f>"Multiple R-squared: "&amp;ROUND('Linear Model'!E41, 4)</f>
-        <v>Multiple R-squared: 0.0109</v>
+        <v>Multiple R-squared: 0.0161</v>
       </c>
       <c r="C13" s="8" t="str">
         <f>"Adjusted R-squared: "&amp;ROUND('Linear Model'!E42, 4)</f>
-        <v>Adjusted R-squared: -0.0097</v>
+        <v>Adjusted R-squared: -0.0044</v>
       </c>
       <c r="D13" s="8"/>
       <c r="E13" s="8"/>
@@ -2702,7 +2765,7 @@
     <row r="14" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B14" s="8" t="str">
         <f>"F-statistic: "&amp;ROUND('Linear Model'!E43, 2)&amp;" on "&amp;'Linear Model'!F43&amp;" and "&amp;'Linear Model'!G43&amp;" DF"</f>
-        <v>F-statistic: 0.53 on 1 and 48 DF</v>
+        <v>F-statistic: 0.78 on 1 and 48 DF</v>
       </c>
       <c r="C14" s="8"/>
       <c r="D14" s="8"/>
@@ -2791,7 +2854,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E54137A-AC86-4C17-97C8-77A96C22EEAE}">
-  <dimension ref="B2:Q57"/>
+  <dimension ref="B2:R59"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="44.109375" customWidth="1"/>
@@ -2821,49 +2884,49 @@
       </c>
       <c r="C4" cm="1">
         <f t="array" ref="C4:Q4">TRANSPOSE(_xll.RScript.Evaluate(B4))</f>
-        <v>-1.4962089497519335</v>
+        <v>3.0791978838770856E-2</v>
       </c>
       <c r="D4">
-        <v>-3.3915554526448028</v>
+        <v>0.10351232004599553</v>
       </c>
       <c r="E4">
-        <v>0.67773592231112656</v>
+        <v>0.11437892297381753</v>
       </c>
       <c r="F4">
-        <v>1.5552069819211933</v>
+        <v>0.27957318459379377</v>
       </c>
       <c r="G4">
-        <v>-1.2253252148789326</v>
+        <v>0.24703052036472256</v>
       </c>
       <c r="H4">
-        <v>-0.95192824683587396</v>
+        <v>0.28799151366236381</v>
       </c>
       <c r="I4">
-        <v>-0.84677764343094009</v>
+        <v>0.1641251131424642</v>
       </c>
       <c r="J4">
-        <v>-0.97594908106725586</v>
+        <v>0.2125209879877088</v>
       </c>
       <c r="K4">
-        <v>2.2907480314435764</v>
+        <v>8.9110367280575392E-2</v>
       </c>
       <c r="L4">
-        <v>-1.6423544299200215</v>
+        <v>0.29343342814550072</v>
       </c>
       <c r="M4">
-        <v>-2.0242010386831493</v>
+        <v>4.8538344019857793E-3</v>
       </c>
       <c r="N4">
-        <v>-1.0441075648736</v>
+        <v>0.18922968109415322</v>
       </c>
       <c r="O4">
-        <v>1.4814564492607833</v>
+        <v>0.1372592664064079</v>
       </c>
       <c r="P4">
-        <v>0.67805394991365231</v>
+        <v>0.10332716144876135</v>
       </c>
       <c r="Q4">
-        <v>0.33821709346702805</v>
+        <v>0.21914586654744209</v>
       </c>
     </row>
     <row r="5" spans="2:17" x14ac:dyDescent="0.3">
@@ -2880,10 +2943,17 @@
         <v>10</v>
       </c>
       <c r="C6" t="str" cm="1">
-        <f t="array" ref="C6">TRANSPOSE(_xll.RScript.Evaluate(B6))</f>
-        <v xml:space="preserve">Exception: Error in model.frame.default(Terms, newdata, na.action = na.action, xlev = object$xlevels) : 
-  'data' must be a data.frame, environment, or list
-</v>
+        <f t="array" ref="C6:F6">TRANSPOSE(_xll.RScript.Evaluate(B6))</f>
+        <v>fit</v>
+      </c>
+      <c r="D6" t="str">
+        <v>se.fit</v>
+      </c>
+      <c r="E6" t="str">
+        <v>df</v>
+      </c>
+      <c r="F6" t="str">
+        <v>residual.scale</v>
       </c>
     </row>
     <row r="7" spans="2:17" ht="28.8" x14ac:dyDescent="0.3">
@@ -2892,9 +2962,7 @@
       </c>
       <c r="C7" t="str" cm="1">
         <f t="array" ref="C7">TRANSPOSE(_xll.RScript.Evaluate(B7))</f>
-        <v xml:space="preserve">Exception: Error in model.frame.default(Terms, newdata, na.action = na.action, xlev = object$xlevels) : 
-  'data' must be a data.frame, environment, or list
-</v>
+        <v>pred.w.plim</v>
       </c>
     </row>
     <row r="8" spans="2:17" ht="28.8" x14ac:dyDescent="0.3">
@@ -2903,9 +2971,7 @@
       </c>
       <c r="C8" t="str" cm="1">
         <f t="array" ref="C8">TRANSPOSE(_xll.RScript.Evaluate(B8))</f>
-        <v xml:space="preserve">Exception: Error in model.frame.default(Terms, newdata, na.action = na.action, xlev = object$xlevels) : 
-  'data' must be a data.frame, environment, or list
-</v>
+        <v>pred.w.clim</v>
       </c>
     </row>
     <row r="9" spans="2:17" ht="28.8" x14ac:dyDescent="0.3">
@@ -2914,21 +2980,20 @@
       </c>
       <c r="C9" t="str" cm="1">
         <f t="array" ref="C9">TRANSPOSE(_xll.RScript.Evaluate(B9))</f>
-        <v xml:space="preserve">Exception: Error: object 'pred.w.clim' not found
-</v>
-      </c>
-    </row>
-    <row r="25" spans="2:17" x14ac:dyDescent="0.3">
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="25" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B25" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="26" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B26" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="27" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B27" t="s">
         <v>16</v>
       </c>
@@ -2937,7 +3002,7 @@
         <v>w</v>
       </c>
     </row>
-    <row r="28" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B28" t="s">
         <v>17</v>
       </c>
@@ -2946,253 +3011,905 @@
         <v>fit</v>
       </c>
     </row>
-    <row r="29" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B29" t="s">
         <v>18</v>
       </c>
       <c r="C29" t="str" cm="1">
         <f t="array" ref="C29">TRANSPOSE(_xll.RScript.Evaluate(B29))</f>
-        <v xml:space="preserve">Exception: Error in eval(extras, data, env) : object 'w' not found
-</v>
-      </c>
-    </row>
-    <row r="30" spans="2:17" x14ac:dyDescent="0.3">
+        <v>wfit</v>
+      </c>
+    </row>
+    <row r="30" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B30" t="s">
         <v>19</v>
       </c>
-      <c r="C30" cm="1">
-        <f t="array" ref="C30:Q32">TRANSPOSE(_xll.RScript.Evaluate(B30))</f>
-        <v>-1.4962089497519335</v>
-      </c>
-      <c r="D30">
-        <v>-3.3915554526448028</v>
-      </c>
-      <c r="E30">
-        <v>0.67773592231112656</v>
-      </c>
-      <c r="F30">
-        <v>1.5552069819211933</v>
-      </c>
-      <c r="G30">
-        <v>-1.2253252148789326</v>
-      </c>
-      <c r="H30">
-        <v>-0.95192824683587396</v>
-      </c>
-      <c r="I30">
-        <v>-0.84677764343094009</v>
-      </c>
-      <c r="J30">
-        <v>-0.97594908106725586</v>
-      </c>
-      <c r="K30">
-        <v>2.2907480314435764</v>
-      </c>
-      <c r="L30">
-        <v>-1.6423544299200215</v>
-      </c>
-      <c r="M30">
-        <v>-2.0242010386831493</v>
-      </c>
-      <c r="N30">
-        <v>-1.0441075648736</v>
-      </c>
-      <c r="O30">
-        <v>1.4814564492607833</v>
-      </c>
-      <c r="P30">
-        <v>0.67805394991365231</v>
-      </c>
-      <c r="Q30">
-        <v>0.33821709346702805</v>
-      </c>
-    </row>
-    <row r="31" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="C31">
-        <v>-4.2502440700749835</v>
+      <c r="C30" t="str" cm="1">
+        <f t="array" ref="C30:R33">TRANSPOSE(_xll.RScript.Evaluate(B30, "DataFrame"))</f>
+        <v>Index</v>
+      </c>
+      <c r="D30" t="str">
+        <v>1</v>
+      </c>
+      <c r="E30" t="str">
+        <v>2</v>
+      </c>
+      <c r="F30" t="str">
+        <v>3</v>
+      </c>
+      <c r="G30" t="str">
+        <v>4</v>
+      </c>
+      <c r="H30" t="str">
+        <v>5</v>
+      </c>
+      <c r="I30" t="str">
+        <v>6</v>
+      </c>
+      <c r="J30" t="str">
+        <v>7</v>
+      </c>
+      <c r="K30" t="str">
+        <v>8</v>
+      </c>
+      <c r="L30" t="str">
+        <v>9</v>
+      </c>
+      <c r="M30" t="str">
+        <v>10</v>
+      </c>
+      <c r="N30" t="str">
+        <v>11</v>
+      </c>
+      <c r="O30" t="str">
+        <v>12</v>
+      </c>
+      <c r="P30" t="str">
+        <v>13</v>
+      </c>
+      <c r="Q30" t="str">
+        <v>14</v>
+      </c>
+      <c r="R30" t="str">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="31" spans="2:18" x14ac:dyDescent="0.3">
+      <c r="C31" t="str">
+        <v>fit</v>
       </c>
       <c r="D31">
-        <v>-6.4147440359458834</v>
+        <v>-0.50015150866533797</v>
       </c>
       <c r="E31">
-        <v>-2.0810146552176167</v>
+        <v>1.8441742009165059</v>
       </c>
       <c r="F31">
-        <v>-1.3029185344471994</v>
+        <v>-2.0305014396555641</v>
       </c>
       <c r="G31">
-        <v>-3.9607414902453839</v>
+        <v>7.3194832127196255E-2</v>
       </c>
       <c r="H31">
-        <v>-3.6740201708791056</v>
+        <v>-0.10620787568641107</v>
       </c>
       <c r="I31">
-        <v>-3.565225467809567</v>
+        <v>0.13916473430692897</v>
       </c>
       <c r="J31">
-        <v>-3.6989893271417484</v>
+        <v>0.69308843162214362</v>
       </c>
       <c r="K31">
-        <v>-0.68909380424313893</v>
+        <v>-0.62919515885903654</v>
       </c>
       <c r="L31">
-        <v>-4.4086368172068973</v>
+        <v>0.86435563075310806</v>
       </c>
       <c r="M31">
-        <v>-4.8295895790485339</v>
+        <v>-0.15590931375969697</v>
       </c>
       <c r="N31">
-        <v>-3.7700725850873864</v>
+        <v>-0.71193379002101553</v>
       </c>
       <c r="O31">
-        <v>-1.3663221106124519</v>
+        <v>1.3573223313036062</v>
       </c>
       <c r="P31">
-        <v>-2.0807229515572621</v>
+        <v>-1.8294545243299636</v>
       </c>
       <c r="Q31">
-        <v>-2.3966042238742369</v>
-      </c>
-    </row>
-    <row r="32" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="C32">
-        <v>1.2578261705711162</v>
+        <v>0.37952818736321364</v>
+      </c>
+      <c r="R31">
+        <v>-1.8283893778739926</v>
+      </c>
+    </row>
+    <row r="32" spans="2:18" x14ac:dyDescent="0.3">
+      <c r="C32" t="str">
+        <v>lwr</v>
       </c>
       <c r="D32">
-        <v>-0.36836686934372187</v>
+        <v>-2.5017912305844789</v>
       </c>
       <c r="E32">
-        <v>3.4364864998398703</v>
+        <v>-0.34846774060965746</v>
       </c>
       <c r="F32">
-        <v>4.4133324982895861</v>
+        <v>-4.1978350594863443</v>
       </c>
       <c r="G32">
-        <v>1.5100910604875186</v>
+        <v>-1.9254671025929748</v>
       </c>
       <c r="H32">
-        <v>1.7701636772073575</v>
+        <v>-2.102181438785407</v>
       </c>
       <c r="I32">
-        <v>1.871670180947687</v>
+        <v>-1.8613131734728652</v>
       </c>
       <c r="J32">
-        <v>1.7470911650072365</v>
+        <v>-1.3399329957316541</v>
       </c>
       <c r="K32">
-        <v>5.2705898671302922</v>
+        <v>-2.6361320175716605</v>
       </c>
       <c r="L32">
-        <v>1.1239279573668539</v>
+        <v>-1.1848355368364003</v>
       </c>
       <c r="M32">
-        <v>0.78118750168223583</v>
+        <v>-2.1517214543468128</v>
       </c>
       <c r="N32">
-        <v>1.6818574553401862</v>
+        <v>-2.7231515305824217</v>
       </c>
       <c r="O32">
-        <v>4.3292350091340186</v>
+        <v>-0.75365001767527318</v>
       </c>
       <c r="P32">
-        <v>3.4368308513845669</v>
+        <v>-3.9629685190365347</v>
       </c>
       <c r="Q32">
-        <v>3.0730384108082931</v>
-      </c>
-    </row>
-    <row r="34" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B34" t="s">
+        <v>-1.6313034857370907</v>
+      </c>
+      <c r="R32">
+        <v>-3.9617330962944353</v>
+      </c>
+    </row>
+    <row r="33" spans="2:18" x14ac:dyDescent="0.3">
+      <c r="C33" t="str">
+        <v>upr</v>
+      </c>
+      <c r="D33">
+        <v>1.5014882132538028</v>
+      </c>
+      <c r="E33">
+        <v>4.0368161424426692</v>
+      </c>
+      <c r="F33">
+        <v>0.13683218017521614</v>
+      </c>
+      <c r="G33">
+        <v>2.0718567668473673</v>
+      </c>
+      <c r="H33">
+        <v>1.889765687412585</v>
+      </c>
+      <c r="I33">
+        <v>2.1396426420867232</v>
+      </c>
+      <c r="J33">
+        <v>2.7261098589759416</v>
+      </c>
+      <c r="K33">
+        <v>1.3777416998535872</v>
+      </c>
+      <c r="L33">
+        <v>2.9135467983426167</v>
+      </c>
+      <c r="M33">
+        <v>1.8399028268274191</v>
+      </c>
+      <c r="N33">
+        <v>1.2992839505403908</v>
+      </c>
+      <c r="O33">
+        <v>3.4682946802824857</v>
+      </c>
+      <c r="P33">
+        <v>0.30405947037660752</v>
+      </c>
+      <c r="Q33">
+        <v>2.3903598604635179</v>
+      </c>
+      <c r="R33">
+        <v>0.3049543405464501</v>
+      </c>
+    </row>
+    <row r="35" spans="2:18" x14ac:dyDescent="0.3">
+      <c r="B35" t="s">
         <v>20</v>
       </c>
-      <c r="C34" t="str" cm="1">
-        <f t="array" ref="C34">TRANSPOSE(_xll.RScript.Evaluate(B34))</f>
-        <v xml:space="preserve">Exception: Error: object 'wfit' not found
-</v>
-      </c>
-    </row>
-    <row r="39" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B39" t="s">
+      <c r="C35" t="str" cm="1">
+        <f t="array" ref="C35:R38">TRANSPOSE(_xll.RScript.Evaluate(B35, "DataFrame"))</f>
+        <v>Index</v>
+      </c>
+      <c r="D35" t="str">
+        <v>1</v>
+      </c>
+      <c r="E35" t="str">
+        <v>2</v>
+      </c>
+      <c r="F35" t="str">
+        <v>3</v>
+      </c>
+      <c r="G35" t="str">
+        <v>4</v>
+      </c>
+      <c r="H35" t="str">
+        <v>5</v>
+      </c>
+      <c r="I35" t="str">
+        <v>6</v>
+      </c>
+      <c r="J35" t="str">
+        <v>7</v>
+      </c>
+      <c r="K35" t="str">
+        <v>8</v>
+      </c>
+      <c r="L35" t="str">
+        <v>9</v>
+      </c>
+      <c r="M35" t="str">
+        <v>10</v>
+      </c>
+      <c r="N35" t="str">
+        <v>11</v>
+      </c>
+      <c r="O35" t="str">
+        <v>12</v>
+      </c>
+      <c r="P35" t="str">
+        <v>13</v>
+      </c>
+      <c r="Q35" t="str">
+        <v>14</v>
+      </c>
+      <c r="R35" t="str">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="36" spans="2:18" x14ac:dyDescent="0.3">
+      <c r="C36" t="str">
+        <v>fit</v>
+      </c>
+      <c r="D36">
+        <v>-0.57016964755585542</v>
+      </c>
+      <c r="E36">
+        <v>1.3561014232058244</v>
+      </c>
+      <c r="F36">
+        <v>-1.8276181275857124</v>
+      </c>
+      <c r="G36">
+        <v>-9.906596717488951E-2</v>
+      </c>
+      <c r="H36">
+        <v>-0.24647647616056406</v>
+      </c>
+      <c r="I36">
+        <v>-4.4860225374419499E-2</v>
+      </c>
+      <c r="J36">
+        <v>0.41028437726612776</v>
+      </c>
+      <c r="K36">
+        <v>-0.67620143708818503</v>
+      </c>
+      <c r="L36">
+        <v>0.55101015172141965</v>
+      </c>
+      <c r="M36">
+        <v>-0.28731484684622299</v>
+      </c>
+      <c r="N36">
+        <v>-0.74418560455703431</v>
+      </c>
+      <c r="O36">
+        <v>0.95606798572377694</v>
+      </c>
+      <c r="P36">
+        <v>-1.6624231398437344</v>
+      </c>
+      <c r="Q36">
+        <v>0.15264013227566586</v>
+      </c>
+      <c r="R36">
+        <v>-1.6615479368820147</v>
+      </c>
+    </row>
+    <row r="37" spans="2:18" x14ac:dyDescent="0.3">
+      <c r="C37" t="str">
+        <v>lwr</v>
+      </c>
+      <c r="D37">
+        <v>-3.3436253984760302</v>
+      </c>
+      <c r="E37">
+        <v>-0.23600258066338919</v>
+      </c>
+      <c r="F37">
+        <v>-3.2808925368840738</v>
+      </c>
+      <c r="G37">
+        <v>-3.1962694413024373</v>
+      </c>
+      <c r="H37">
+        <v>-3.356359799501992</v>
+      </c>
+      <c r="I37">
+        <v>-3.1077716883273792</v>
+      </c>
+      <c r="J37">
+        <v>-2.0402319711770271</v>
+      </c>
+      <c r="K37">
+        <v>-3.2845789396344802</v>
+      </c>
+      <c r="L37">
+        <v>-1.6997862553342813</v>
+      </c>
+      <c r="M37">
+        <v>-3.3792084538918257</v>
+      </c>
+      <c r="N37">
+        <v>-3.245083767779624</v>
+      </c>
+      <c r="O37">
+        <v>-0.86392298660823552</v>
+      </c>
+      <c r="P37">
+        <v>-3.1917202263546365</v>
+      </c>
+      <c r="Q37">
+        <v>-2.6855786894118201</v>
+      </c>
+      <c r="R37">
+        <v>-3.1913117871725172</v>
+      </c>
+    </row>
+    <row r="38" spans="2:18" x14ac:dyDescent="0.3">
+      <c r="C38" t="str">
+        <v>upr</v>
+      </c>
+      <c r="D38">
+        <v>2.2032861033643192</v>
+      </c>
+      <c r="E38">
+        <v>2.9482054270750382</v>
+      </c>
+      <c r="F38">
+        <v>-0.37434371828735102</v>
+      </c>
+      <c r="G38">
+        <v>2.9981375069526583</v>
+      </c>
+      <c r="H38">
+        <v>2.8634068471808636</v>
+      </c>
+      <c r="I38">
+        <v>3.0180512375785402</v>
+      </c>
+      <c r="J38">
+        <v>2.8608007257092831</v>
+      </c>
+      <c r="K38">
+        <v>1.9321760654581102</v>
+      </c>
+      <c r="L38">
+        <v>2.8018065587771206</v>
+      </c>
+      <c r="M38">
+        <v>2.8045787601993792</v>
+      </c>
+      <c r="N38">
+        <v>1.7567125586655552</v>
+      </c>
+      <c r="O38">
+        <v>2.7760589580557893</v>
+      </c>
+      <c r="P38">
+        <v>-0.13312605333283201</v>
+      </c>
+      <c r="Q38">
+        <v>2.9908589539631518</v>
+      </c>
+      <c r="R38">
+        <v>-0.13178408659151253</v>
+      </c>
+    </row>
+    <row r="40" spans="2:18" x14ac:dyDescent="0.3">
+      <c r="B40" t="s">
         <v>21</v>
       </c>
-      <c r="C39" t="str" cm="1">
-        <f t="array" ref="C39">TRANSPOSE(_xll.RScript.Evaluate(B39))</f>
-        <v xml:space="preserve">Exception: Error: object 'wfit' not found
-</v>
-      </c>
-    </row>
-    <row r="43" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B43" t="s">
+      <c r="C40" t="str" cm="1">
+        <f t="array" ref="C40:P43">TRANSPOSE(_xll.RScript.Evaluate(B40, "DataFrame"))</f>
+        <v>Index</v>
+      </c>
+      <c r="D40" t="str">
+        <v>1</v>
+      </c>
+      <c r="E40" t="str">
+        <v>2</v>
+      </c>
+      <c r="F40" t="str">
+        <v>3</v>
+      </c>
+      <c r="G40" t="str">
+        <v>4</v>
+      </c>
+      <c r="H40" t="str">
+        <v>5</v>
+      </c>
+      <c r="I40" t="str">
+        <v>6</v>
+      </c>
+      <c r="J40" t="str">
+        <v>7</v>
+      </c>
+      <c r="K40" t="str">
+        <v>8</v>
+      </c>
+      <c r="L40" t="str">
+        <v>9</v>
+      </c>
+      <c r="M40" t="str">
+        <v>10</v>
+      </c>
+      <c r="N40" t="str">
+        <v>11</v>
+      </c>
+      <c r="O40" t="str">
+        <v>12</v>
+      </c>
+      <c r="P40" t="str">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="41" spans="2:18" x14ac:dyDescent="0.3">
+      <c r="C41" t="str">
+        <v>fit</v>
+      </c>
+      <c r="D41">
+        <v>-2.3717346511827562</v>
+      </c>
+      <c r="E41">
+        <v>-2.0082830615751712</v>
+      </c>
+      <c r="F41">
+        <v>-1.6448314719675858</v>
+      </c>
+      <c r="G41">
+        <v>-1.2813798823600004</v>
+      </c>
+      <c r="H41">
+        <v>-0.91792829275241505</v>
+      </c>
+      <c r="I41">
+        <v>-0.55447670314482966</v>
+      </c>
+      <c r="J41">
+        <v>-0.19102511353724438</v>
+      </c>
+      <c r="K41">
+        <v>0.17242647607034095</v>
+      </c>
+      <c r="L41">
+        <v>0.53587806567792629</v>
+      </c>
+      <c r="M41">
+        <v>0.89932965528551156</v>
+      </c>
+      <c r="N41">
+        <v>1.2627812448930968</v>
+      </c>
+      <c r="O41">
+        <v>1.6262328345006822</v>
+      </c>
+      <c r="P41">
+        <v>1.9896844241082676</v>
+      </c>
+    </row>
+    <row r="42" spans="2:18" x14ac:dyDescent="0.3">
+      <c r="C42" t="str">
+        <v>lwr</v>
+      </c>
+      <c r="D42">
+        <v>-5.5843909291607634</v>
+      </c>
+      <c r="E42">
+        <v>-5.1879906252697197</v>
+      </c>
+      <c r="F42">
+        <v>-4.7983751565659079</v>
+      </c>
+      <c r="G42">
+        <v>-4.4157144370290506</v>
+      </c>
+      <c r="H42">
+        <v>-4.0401368348558613</v>
+      </c>
+      <c r="I42">
+        <v>-3.6717250105537627</v>
+      </c>
+      <c r="J42">
+        <v>-3.3105131467844973</v>
+      </c>
+      <c r="K42">
+        <v>-2.9564857820427881</v>
+      </c>
+      <c r="L42">
+        <v>-2.6095783397165624</v>
+      </c>
+      <c r="M42">
+        <v>-2.2696793108382289</v>
+      </c>
+      <c r="N42">
+        <v>-1.93663392141104</v>
+      </c>
+      <c r="O42">
+        <v>-1.6102490108446657</v>
+      </c>
+      <c r="P42">
+        <v>-1.2902987792011578</v>
+      </c>
+    </row>
+    <row r="43" spans="2:18" x14ac:dyDescent="0.3">
+      <c r="C43" t="str">
+        <v>upr</v>
+      </c>
+      <c r="D43">
+        <v>0.84092162679525151</v>
+      </c>
+      <c r="E43">
+        <v>1.1714245021193772</v>
+      </c>
+      <c r="F43">
+        <v>1.5087122126307362</v>
+      </c>
+      <c r="G43">
+        <v>1.8529546723090498</v>
+      </c>
+      <c r="H43">
+        <v>2.2042802493510316</v>
+      </c>
+      <c r="I43">
+        <v>2.5627716042641033</v>
+      </c>
+      <c r="J43">
+        <v>2.9284629197100087</v>
+      </c>
+      <c r="K43">
+        <v>3.3013387341834703</v>
+      </c>
+      <c r="L43">
+        <v>3.6813344710724145</v>
+      </c>
+      <c r="M43">
+        <v>4.0683386214092518</v>
+      </c>
+      <c r="N43">
+        <v>4.4621964111972332</v>
+      </c>
+      <c r="O43">
+        <v>4.8627146798460306</v>
+      </c>
+      <c r="P43">
+        <v>5.269667627417693</v>
+      </c>
+    </row>
+    <row r="45" spans="2:18" x14ac:dyDescent="0.3">
+      <c r="B45" t="s">
         <v>22</v>
       </c>
-      <c r="C43" t="str" cm="1">
-        <f t="array" ref="C43">TRANSPOSE(_xll.RScript.Evaluate(B43))</f>
-        <v xml:space="preserve">Exception: Error: object 'wfit' not found
-</v>
-      </c>
-    </row>
-    <row r="48" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B48" t="s">
+      <c r="C45" cm="1">
+        <f t="array" ref="C45:O47">TRANSPOSE(_xll.RScript.Evaluate(B45))</f>
+        <v>0.49266116902112089</v>
+      </c>
+      <c r="D45">
+        <v>0.39401981488196058</v>
+      </c>
+      <c r="E45">
+        <v>0.29537846074280033</v>
+      </c>
+      <c r="F45">
+        <v>0.19673710660364008</v>
+      </c>
+      <c r="G45">
+        <v>9.809575246447981E-2</v>
+      </c>
+      <c r="H45">
+        <v>-5.4560167468045706E-4</v>
+      </c>
+      <c r="I45">
+        <v>-9.9186955813840724E-2</v>
+      </c>
+      <c r="J45">
+        <v>-0.19782830995300099</v>
+      </c>
+      <c r="K45">
+        <v>-0.29646966409216124</v>
+      </c>
+      <c r="L45">
+        <v>-0.39511101823132155</v>
+      </c>
+      <c r="M45">
+        <v>-0.49375237237048181</v>
+      </c>
+      <c r="N45">
+        <v>-0.59239372650964206</v>
+      </c>
+      <c r="O45">
+        <v>-0.69103508064880237</v>
+      </c>
+    </row>
+    <row r="46" spans="2:18" x14ac:dyDescent="0.3">
+      <c r="C46">
+        <v>-4.9267634248881365</v>
+      </c>
+      <c r="D46">
+        <v>-4.4244060641645868</v>
+      </c>
+      <c r="E46">
+        <v>-4.2430892526574446</v>
+      </c>
+      <c r="F46">
+        <v>-4.7248537930438941</v>
+      </c>
+      <c r="G46">
+        <v>-6.6156983461381467</v>
+      </c>
+      <c r="H46">
+        <v>-13.127545891525109</v>
+      </c>
+      <c r="I46" t="e">
+        <v>#NUM!</v>
+      </c>
+      <c r="J46">
+        <v>-13.43946651803113</v>
+      </c>
+      <c r="K46">
+        <v>-7.4463453865249747</v>
+      </c>
+      <c r="L46">
+        <v>-6.1649112275277815</v>
+      </c>
+      <c r="M46">
+        <v>-6.2111882033336796</v>
+      </c>
+      <c r="N46">
+        <v>-6.7836340765018965</v>
+      </c>
+      <c r="O46">
+        <v>-7.5835845271509159</v>
+      </c>
+    </row>
+    <row r="47" spans="2:18" x14ac:dyDescent="0.3">
+      <c r="C47">
+        <v>5.9120857629303778</v>
+      </c>
+      <c r="D47">
+        <v>5.2124456939285073</v>
+      </c>
+      <c r="E47">
+        <v>4.8338461741430461</v>
+      </c>
+      <c r="F47">
+        <v>5.1183280062511747</v>
+      </c>
+      <c r="G47">
+        <v>6.8118898510671064</v>
+      </c>
+      <c r="H47">
+        <v>13.126454688175748</v>
+      </c>
+      <c r="I47" t="e">
+        <v>#NUM!</v>
+      </c>
+      <c r="J47">
+        <v>13.043809898125128</v>
+      </c>
+      <c r="K47">
+        <v>6.8534060583406529</v>
+      </c>
+      <c r="L47">
+        <v>5.3746891910651389</v>
+      </c>
+      <c r="M47">
+        <v>5.2236834585927161</v>
+      </c>
+      <c r="N47">
+        <v>5.5988466234826122</v>
+      </c>
+      <c r="O47">
+        <v>6.2015143658533107</v>
+      </c>
+    </row>
+    <row r="50" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="B50" t="s">
         <v>23</v>
       </c>
-      <c r="C48" t="str" cm="1">
-        <f t="array" ref="C48">TRANSPOSE(_xll.RScript.Evaluate(B48))</f>
-        <v xml:space="preserve">Exception: Error: object 'wfit' not found
-</v>
-      </c>
-    </row>
-    <row r="52" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B52" t="s">
+      <c r="C50" cm="1">
+        <f t="array" ref="C50:O52">TRANSPOSE(_xll.RScript.Evaluate(B50))</f>
+        <v>0.49266116902112089</v>
+      </c>
+      <c r="D50">
+        <v>0.39401981488196058</v>
+      </c>
+      <c r="E50">
+        <v>0.29537846074280033</v>
+      </c>
+      <c r="F50">
+        <v>0.19673710660364008</v>
+      </c>
+      <c r="G50">
+        <v>9.809575246447981E-2</v>
+      </c>
+      <c r="H50">
+        <v>-5.4560167468045706E-4</v>
+      </c>
+      <c r="I50">
+        <v>-9.9186955813840724E-2</v>
+      </c>
+      <c r="J50">
+        <v>-0.19782830995300099</v>
+      </c>
+      <c r="K50">
+        <v>-0.29646966409216124</v>
+      </c>
+      <c r="L50">
+        <v>-0.39511101823132155</v>
+      </c>
+      <c r="M50">
+        <v>-0.49375237237048181</v>
+      </c>
+      <c r="N50">
+        <v>-0.59239372650964206</v>
+      </c>
+      <c r="O50">
+        <v>-0.69103508064880237</v>
+      </c>
+    </row>
+    <row r="51" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="C51">
+        <v>-4.9267634248881365</v>
+      </c>
+      <c r="D51">
+        <v>-4.4244060641645868</v>
+      </c>
+      <c r="E51">
+        <v>-4.2430892526574446</v>
+      </c>
+      <c r="F51">
+        <v>-4.7248537930438941</v>
+      </c>
+      <c r="G51">
+        <v>-6.6156983461381467</v>
+      </c>
+      <c r="H51">
+        <v>-13.127545891525109</v>
+      </c>
+      <c r="I51" t="e">
+        <v>#NUM!</v>
+      </c>
+      <c r="J51">
+        <v>-13.43946651803113</v>
+      </c>
+      <c r="K51">
+        <v>-7.4463453865249747</v>
+      </c>
+      <c r="L51">
+        <v>-6.1649112275277815</v>
+      </c>
+      <c r="M51">
+        <v>-6.2111882033336796</v>
+      </c>
+      <c r="N51">
+        <v>-6.7836340765018965</v>
+      </c>
+      <c r="O51">
+        <v>-7.5835845271509159</v>
+      </c>
+    </row>
+    <row r="52" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="C52">
+        <v>5.9120857629303778</v>
+      </c>
+      <c r="D52">
+        <v>5.2124456939285073</v>
+      </c>
+      <c r="E52">
+        <v>4.8338461741430461</v>
+      </c>
+      <c r="F52">
+        <v>5.1183280062511747</v>
+      </c>
+      <c r="G52">
+        <v>6.8118898510671064</v>
+      </c>
+      <c r="H52">
+        <v>13.126454688175748</v>
+      </c>
+      <c r="I52" t="e">
+        <v>#NUM!</v>
+      </c>
+      <c r="J52">
+        <v>13.043809898125128</v>
+      </c>
+      <c r="K52">
+        <v>6.8534060583406529</v>
+      </c>
+      <c r="L52">
+        <v>5.3746891910651389</v>
+      </c>
+      <c r="M52">
+        <v>5.2236834585927161</v>
+      </c>
+      <c r="N52">
+        <v>5.5988466234826122</v>
+      </c>
+      <c r="O52">
+        <v>6.2015143658533107</v>
+      </c>
+    </row>
+    <row r="54" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="B54" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="53" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B53" t="s">
+    <row r="55" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="B55" t="s">
         <v>25</v>
-      </c>
-      <c r="C53" t="str" cm="1">
-        <f t="array" ref="C53">TRANSPOSE(_xll.RScript.Evaluate(B53))</f>
-        <v>npk.aov</v>
-      </c>
-    </row>
-    <row r="54" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B54" t="s">
-        <v>28</v>
-      </c>
-      <c r="C54" t="str" cm="1">
-        <f t="array" ref="C54">TRANSPOSE(_xll.RScript.Evaluate(B54))</f>
-        <v xml:space="preserve">Exception: Error: object 'npk.aov' not found
-</v>
-      </c>
-    </row>
-    <row r="55" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B55" t="s">
-        <v>29</v>
       </c>
       <c r="C55" t="str" cm="1">
         <f t="array" ref="C55">TRANSPOSE(_xll.RScript.Evaluate(B55))</f>
-        <v xml:space="preserve">Exception: Error: object 'npk.aov' not found
-</v>
-      </c>
-    </row>
-    <row r="56" spans="2:3" x14ac:dyDescent="0.3">
+        <v>npk.aov</v>
+      </c>
+    </row>
+    <row r="56" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B56" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C56" t="str" cm="1">
         <f t="array" ref="C56">TRANSPOSE(_xll.RScript.Evaluate(B56))</f>
-        <v xml:space="preserve">Exception: Error: object 'npk.aov' not found
-</v>
-      </c>
-    </row>
-    <row r="57" spans="2:3" x14ac:dyDescent="0.3">
+        <v>termL</v>
+      </c>
+    </row>
+    <row r="57" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B57" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C57" t="str" cm="1">
         <f t="array" ref="C57">TRANSPOSE(_xll.RScript.Evaluate(B57))</f>
-        <v xml:space="preserve">Exception: Error in pt[, 1:4] : object of type 'closure' is not subsettable
-</v>
+        <v>pt</v>
+      </c>
+    </row>
+    <row r="58" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="B58" t="s">
+        <v>26</v>
+      </c>
+      <c r="C58" t="str" cm="1">
+        <f t="array" ref="C58">TRANSPOSE(_xll.RScript.Evaluate(B58))</f>
+        <v>pt.</v>
+      </c>
+    </row>
+    <row r="59" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="B59" t="s">
+        <v>27</v>
+      </c>
+      <c r="C59" t="str" cm="1">
+        <f t="array" ref="C59">TRANSPOSE(_xll.RScript.Evaluate(B59))</f>
+        <v>OK</v>
       </c>
     </row>
   </sheetData>

</xml_diff>